<commit_message>
Updated architecture to connect benchmarks to full run
</commit_message>
<xml_diff>
--- a/docs/KH-literature/Literature_Review.xlsx
+++ b/docs/KH-literature/Literature_Review.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\QuantumHPC\docs\KH-literature\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\QuantumHPC\docs\KH-literature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CAA56C6-92EA-4CF1-8FD2-520B3FED719D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FE4E522-F39C-44B4-ACB1-E6141D45F315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kyle" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="290">
   <si>
     <t>Type of Survey</t>
   </si>
@@ -926,6 +926,12 @@
   <si>
     <t>https://www.psc.edu/resources/bridges-2/user-guide/</t>
   </si>
+  <si>
+    <t>Havlicek et al</t>
+  </si>
+  <si>
+    <t>IBM ZZFeatureMap Docs</t>
+  </si>
 </sst>
 </file>
 
@@ -1070,15 +1076,15 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1300,6 +1306,9 @@
   </sheetPr>
   <dimension ref="A1:AH975"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="21.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="76.5">
       <c r="A1" s="10" t="s">
@@ -1421,12 +1430,12 @@
       <c r="T2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="U2" s="14" t="s">
+      <c r="U2" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="V2" s="15"/>
-      <c r="W2" s="15"/>
-      <c r="X2" s="15"/>
+      <c r="V2" s="17"/>
+      <c r="W2" s="17"/>
+      <c r="X2" s="17"/>
       <c r="Y2" s="3"/>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
@@ -1539,12 +1548,12 @@
       <c r="T4" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="U4" s="14" t="s">
+      <c r="U4" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="V4" s="15"/>
-      <c r="W4" s="15"/>
-      <c r="X4" s="15"/>
+      <c r="V4" s="17"/>
+      <c r="W4" s="17"/>
+      <c r="X4" s="17"/>
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
       <c r="AA4" s="3"/>
@@ -1598,12 +1607,12 @@
       <c r="T5" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="U5" s="14" t="s">
+      <c r="U5" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="V5" s="15"/>
-      <c r="W5" s="15"/>
-      <c r="X5" s="15"/>
+      <c r="V5" s="17"/>
+      <c r="W5" s="17"/>
+      <c r="X5" s="17"/>
       <c r="Y5" s="3"/>
       <c r="Z5" s="3"/>
       <c r="AA5" s="3"/>
@@ -1672,12 +1681,18 @@
       <c r="AH6" s="3"/>
     </row>
     <row r="7" spans="1:34" ht="15.75" customHeight="1">
-      <c r="U7" s="19" t="s">
+      <c r="A7" t="s">
+        <v>289</v>
+      </c>
+      <c r="U7" s="14" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="8" spans="1:34" ht="15.75" customHeight="1">
-      <c r="U8" s="20" t="s">
+      <c r="A8" t="s">
+        <v>288</v>
+      </c>
+      <c r="U8" s="15" t="s">
         <v>283</v>
       </c>
     </row>
@@ -1720,7 +1735,7 @@
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
-      <c r="U9" s="19" t="s">
+      <c r="U9" s="14" t="s">
         <v>284</v>
       </c>
       <c r="V9" s="3"/>
@@ -1776,7 +1791,7 @@
       <c r="R10" s="3"/>
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
-      <c r="U10" s="19" t="s">
+      <c r="U10" s="14" t="s">
         <v>285</v>
       </c>
       <c r="V10" s="3"/>
@@ -1832,7 +1847,7 @@
       <c r="R11" s="3"/>
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
-      <c r="U11" s="19" t="s">
+      <c r="U11" s="14" t="s">
         <v>286</v>
       </c>
       <c r="V11" s="3"/>
@@ -1888,7 +1903,7 @@
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
-      <c r="U12" s="19" t="s">
+      <c r="U12" s="14" t="s">
         <v>287</v>
       </c>
       <c r="V12" s="3"/>
@@ -35738,12 +35753,12 @@
       <c r="M2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="16" t="s">
+      <c r="N2" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="O2" s="15"/>
-      <c r="P2" s="15"/>
-      <c r="Q2" s="15"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
@@ -35795,12 +35810,12 @@
       <c r="M3" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="N3" s="16" t="s">
+      <c r="N3" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="O3" s="15"/>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
+      <c r="O3" s="17"/>
+      <c r="P3" s="17"/>
+      <c r="Q3" s="17"/>
       <c r="R3" s="3"/>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
@@ -35852,12 +35867,12 @@
       <c r="M4" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="N4" s="16" t="s">
+      <c r="N4" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
-      <c r="Q4" s="15"/>
+      <c r="O4" s="17"/>
+      <c r="P4" s="17"/>
+      <c r="Q4" s="17"/>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
@@ -35909,12 +35924,12 @@
       <c r="M5" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="N5" s="16" t="s">
+      <c r="N5" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
+      <c r="O5" s="17"/>
+      <c r="P5" s="17"/>
+      <c r="Q5" s="17"/>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
@@ -35966,12 +35981,12 @@
       <c r="M6" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="16" t="s">
+      <c r="N6" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
@@ -36023,10 +36038,10 @@
       <c r="M7" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="N7" s="17"/>
-      <c r="O7" s="15"/>
-      <c r="P7" s="15"/>
-      <c r="Q7" s="15"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="17"/>
+      <c r="P7" s="17"/>
+      <c r="Q7" s="17"/>
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
@@ -36078,10 +36093,10 @@
       <c r="M8" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="N8" s="17"/>
-      <c r="O8" s="15"/>
-      <c r="P8" s="15"/>
-      <c r="Q8" s="15"/>
+      <c r="N8" s="18"/>
+      <c r="O8" s="17"/>
+      <c r="P8" s="17"/>
+      <c r="Q8" s="17"/>
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
       <c r="T8" s="3"/>
@@ -36133,10 +36148,10 @@
       <c r="M9" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="N9" s="17"/>
-      <c r="O9" s="15"/>
-      <c r="P9" s="15"/>
-      <c r="Q9" s="15"/>
+      <c r="N9" s="18"/>
+      <c r="O9" s="17"/>
+      <c r="P9" s="17"/>
+      <c r="Q9" s="17"/>
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
@@ -36188,10 +36203,10 @@
       <c r="M10" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="N10" s="17"/>
-      <c r="O10" s="15"/>
-      <c r="P10" s="15"/>
-      <c r="Q10" s="15"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="17"/>
+      <c r="P10" s="17"/>
+      <c r="Q10" s="17"/>
       <c r="R10" s="3"/>
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
@@ -36243,10 +36258,10 @@
       <c r="M11" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="N11" s="17"/>
-      <c r="O11" s="15"/>
-      <c r="P11" s="15"/>
-      <c r="Q11" s="15"/>
+      <c r="N11" s="18"/>
+      <c r="O11" s="17"/>
+      <c r="P11" s="17"/>
+      <c r="Q11" s="17"/>
       <c r="R11" s="3"/>
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
@@ -36298,10 +36313,10 @@
       <c r="M12" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="N12" s="17"/>
-      <c r="O12" s="15"/>
-      <c r="P12" s="15"/>
-      <c r="Q12" s="15"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="17"/>
+      <c r="P12" s="17"/>
+      <c r="Q12" s="17"/>
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
@@ -36353,10 +36368,10 @@
       <c r="M13" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="N13" s="17"/>
-      <c r="O13" s="15"/>
-      <c r="P13" s="15"/>
-      <c r="Q13" s="15"/>
+      <c r="N13" s="18"/>
+      <c r="O13" s="17"/>
+      <c r="P13" s="17"/>
+      <c r="Q13" s="17"/>
       <c r="R13" s="3"/>
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
@@ -36408,10 +36423,10 @@
       <c r="M14" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="N14" s="17"/>
-      <c r="O14" s="15"/>
-      <c r="P14" s="15"/>
-      <c r="Q14" s="15"/>
+      <c r="N14" s="18"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
@@ -36463,10 +36478,10 @@
       <c r="M15" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="N15" s="17"/>
-      <c r="O15" s="15"/>
-      <c r="P15" s="15"/>
-      <c r="Q15" s="15"/>
+      <c r="N15" s="18"/>
+      <c r="O15" s="17"/>
+      <c r="P15" s="17"/>
+      <c r="Q15" s="17"/>
       <c r="R15" s="3"/>
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
@@ -36518,10 +36533,10 @@
       <c r="M16" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="N16" s="17"/>
-      <c r="O16" s="15"/>
-      <c r="P16" s="15"/>
-      <c r="Q16" s="15"/>
+      <c r="N16" s="18"/>
+      <c r="O16" s="17"/>
+      <c r="P16" s="17"/>
+      <c r="Q16" s="17"/>
       <c r="R16" s="3"/>
       <c r="S16" s="3"/>
       <c r="T16" s="3"/>
@@ -36573,10 +36588,10 @@
       <c r="M17" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="N17" s="17"/>
-      <c r="O17" s="15"/>
-      <c r="P17" s="15"/>
-      <c r="Q17" s="15"/>
+      <c r="N17" s="18"/>
+      <c r="O17" s="17"/>
+      <c r="P17" s="17"/>
+      <c r="Q17" s="17"/>
       <c r="R17" s="3"/>
       <c r="S17" s="3"/>
       <c r="T17" s="3"/>
@@ -36601,11 +36616,11 @@
       <c r="D18" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
       <c r="H18" s="3"/>
       <c r="I18" s="4" t="s">
         <v>22</v>
@@ -36622,10 +36637,10 @@
       <c r="M18" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="N18" s="17"/>
-      <c r="O18" s="15"/>
-      <c r="P18" s="15"/>
-      <c r="Q18" s="15"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="17"/>
+      <c r="P18" s="17"/>
+      <c r="Q18" s="17"/>
       <c r="R18" s="3"/>
       <c r="S18" s="3"/>
       <c r="T18" s="3"/>
@@ -36677,10 +36692,10 @@
       <c r="M19" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="N19" s="17"/>
-      <c r="O19" s="15"/>
-      <c r="P19" s="15"/>
-      <c r="Q19" s="15"/>
+      <c r="N19" s="18"/>
+      <c r="O19" s="17"/>
+      <c r="P19" s="17"/>
+      <c r="Q19" s="17"/>
       <c r="R19" s="3"/>
       <c r="S19" s="3"/>
       <c r="T19" s="3"/>
@@ -36732,10 +36747,10 @@
       <c r="M20" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="N20" s="17"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15"/>
-      <c r="Q20" s="15"/>
+      <c r="N20" s="18"/>
+      <c r="O20" s="17"/>
+      <c r="P20" s="17"/>
+      <c r="Q20" s="17"/>
       <c r="R20" s="3"/>
       <c r="S20" s="3"/>
       <c r="T20" s="3"/>
@@ -36787,10 +36802,10 @@
       <c r="M21" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="N21" s="17"/>
-      <c r="O21" s="15"/>
-      <c r="P21" s="15"/>
-      <c r="Q21" s="15"/>
+      <c r="N21" s="18"/>
+      <c r="O21" s="17"/>
+      <c r="P21" s="17"/>
+      <c r="Q21" s="17"/>
       <c r="R21" s="3"/>
       <c r="S21" s="3"/>
       <c r="T21" s="3"/>
@@ -36842,10 +36857,10 @@
       <c r="M22" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="N22" s="17"/>
-      <c r="O22" s="15"/>
-      <c r="P22" s="15"/>
-      <c r="Q22" s="15"/>
+      <c r="N22" s="18"/>
+      <c r="O22" s="17"/>
+      <c r="P22" s="17"/>
+      <c r="Q22" s="17"/>
       <c r="R22" s="3"/>
       <c r="S22" s="3"/>
       <c r="T22" s="3"/>
@@ -36897,10 +36912,10 @@
       <c r="M23" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="N23" s="17"/>
-      <c r="O23" s="15"/>
-      <c r="P23" s="15"/>
-      <c r="Q23" s="15"/>
+      <c r="N23" s="18"/>
+      <c r="O23" s="17"/>
+      <c r="P23" s="17"/>
+      <c r="Q23" s="17"/>
       <c r="R23" s="3"/>
       <c r="S23" s="3"/>
       <c r="T23" s="3"/>
@@ -36952,10 +36967,10 @@
       <c r="M24" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="N24" s="17"/>
-      <c r="O24" s="15"/>
-      <c r="P24" s="15"/>
-      <c r="Q24" s="15"/>
+      <c r="N24" s="18"/>
+      <c r="O24" s="17"/>
+      <c r="P24" s="17"/>
+      <c r="Q24" s="17"/>
       <c r="R24" s="3"/>
       <c r="S24" s="3"/>
       <c r="T24" s="3"/>
@@ -37007,10 +37022,10 @@
       <c r="M25" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="N25" s="17"/>
-      <c r="O25" s="15"/>
-      <c r="P25" s="15"/>
-      <c r="Q25" s="15"/>
+      <c r="N25" s="18"/>
+      <c r="O25" s="17"/>
+      <c r="P25" s="17"/>
+      <c r="Q25" s="17"/>
       <c r="R25" s="3"/>
       <c r="S25" s="3"/>
       <c r="T25" s="3"/>
@@ -37062,10 +37077,10 @@
       <c r="M26" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="N26" s="17"/>
-      <c r="O26" s="15"/>
-      <c r="P26" s="15"/>
-      <c r="Q26" s="15"/>
+      <c r="N26" s="18"/>
+      <c r="O26" s="17"/>
+      <c r="P26" s="17"/>
+      <c r="Q26" s="17"/>
       <c r="R26" s="3"/>
       <c r="S26" s="3"/>
       <c r="T26" s="3"/>
@@ -37117,10 +37132,10 @@
       <c r="M27" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="N27" s="17"/>
-      <c r="O27" s="15"/>
-      <c r="P27" s="15"/>
-      <c r="Q27" s="15"/>
+      <c r="N27" s="18"/>
+      <c r="O27" s="17"/>
+      <c r="P27" s="17"/>
+      <c r="Q27" s="17"/>
       <c r="R27" s="3"/>
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
@@ -37172,10 +37187,10 @@
       <c r="M28" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="N28" s="17"/>
-      <c r="O28" s="15"/>
-      <c r="P28" s="15"/>
-      <c r="Q28" s="15"/>
+      <c r="N28" s="18"/>
+      <c r="O28" s="17"/>
+      <c r="P28" s="17"/>
+      <c r="Q28" s="17"/>
       <c r="R28" s="3"/>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
@@ -37227,10 +37242,10 @@
       <c r="M29" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="N29" s="17"/>
-      <c r="O29" s="15"/>
-      <c r="P29" s="15"/>
-      <c r="Q29" s="15"/>
+      <c r="N29" s="18"/>
+      <c r="O29" s="17"/>
+      <c r="P29" s="17"/>
+      <c r="Q29" s="17"/>
       <c r="R29" s="3"/>
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
@@ -37282,10 +37297,10 @@
       <c r="M30" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="N30" s="17"/>
-      <c r="O30" s="15"/>
-      <c r="P30" s="15"/>
-      <c r="Q30" s="15"/>
+      <c r="N30" s="18"/>
+      <c r="O30" s="17"/>
+      <c r="P30" s="17"/>
+      <c r="Q30" s="17"/>
       <c r="R30" s="3"/>
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
@@ -37337,10 +37352,10 @@
       <c r="M31" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="N31" s="17"/>
-      <c r="O31" s="15"/>
-      <c r="P31" s="15"/>
-      <c r="Q31" s="15"/>
+      <c r="N31" s="18"/>
+      <c r="O31" s="17"/>
+      <c r="P31" s="17"/>
+      <c r="Q31" s="17"/>
       <c r="R31" s="3"/>
       <c r="S31" s="3"/>
       <c r="T31" s="3"/>
@@ -65455,6 +65470,26 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="N2:Q2"/>
+    <mergeCell ref="N3:Q3"/>
+    <mergeCell ref="N4:Q4"/>
+    <mergeCell ref="N5:Q5"/>
+    <mergeCell ref="N6:Q6"/>
+    <mergeCell ref="N7:Q7"/>
+    <mergeCell ref="N8:Q8"/>
+    <mergeCell ref="N9:Q9"/>
+    <mergeCell ref="N10:Q10"/>
+    <mergeCell ref="N11:Q11"/>
+    <mergeCell ref="N12:Q12"/>
+    <mergeCell ref="N13:Q13"/>
+    <mergeCell ref="N14:Q14"/>
+    <mergeCell ref="N15:Q15"/>
+    <mergeCell ref="N16:Q16"/>
+    <mergeCell ref="N17:Q17"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="N18:Q18"/>
+    <mergeCell ref="N19:Q19"/>
+    <mergeCell ref="N20:Q20"/>
     <mergeCell ref="N21:Q21"/>
     <mergeCell ref="N29:Q29"/>
     <mergeCell ref="N30:Q30"/>
@@ -65466,26 +65501,6 @@
     <mergeCell ref="N26:Q26"/>
     <mergeCell ref="N27:Q27"/>
     <mergeCell ref="N28:Q28"/>
-    <mergeCell ref="N17:Q17"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="N18:Q18"/>
-    <mergeCell ref="N19:Q19"/>
-    <mergeCell ref="N20:Q20"/>
-    <mergeCell ref="N12:Q12"/>
-    <mergeCell ref="N13:Q13"/>
-    <mergeCell ref="N14:Q14"/>
-    <mergeCell ref="N15:Q15"/>
-    <mergeCell ref="N16:Q16"/>
-    <mergeCell ref="N7:Q7"/>
-    <mergeCell ref="N8:Q8"/>
-    <mergeCell ref="N9:Q9"/>
-    <mergeCell ref="N10:Q10"/>
-    <mergeCell ref="N11:Q11"/>
-    <mergeCell ref="N2:Q2"/>
-    <mergeCell ref="N3:Q3"/>
-    <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="N5:Q5"/>
-    <mergeCell ref="N6:Q6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>

</xml_diff>